<commit_message>
Fix DishToday crashes and faded controls; focus nav on DishToday and Parties.
Hide Sauce/Drink/MyFavorite for now, clear recipe state on Another One, fix React.Fragment crash on header ingredients, and add a QA checklist with automated run notes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/recipes/excel/Europe.xlsx
+++ b/src/recipes/excel/Europe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashleynordahl/Documents/FoodToday/src/recipes/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB63C2B8-635B-6C4D-A80E-1C82038E1584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AD19DE-F70C-444D-BC15-47189E9DB64B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2680" yWindow="2040" windowWidth="19180" windowHeight="14360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6220,13 +6220,13 @@
         <v>96</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>167</v>
+        <v>40</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>168</v>
+        <v>41</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>169</v>
+        <v>42</v>
       </c>
       <c r="Q23" s="1" t="s">
         <v>60</v>
@@ -6283,7 +6283,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="136">
+    <row r="24" spans="1:37" ht="153">
       <c r="A24" s="1" t="s">
         <v>98</v>
       </c>

</xml_diff>